<commit_message>
Add eval sheets for 楊玉鳳 and 鍾欣芳; update roles in script
- 楊玉鳳: field_worker → section_chief（副課長）
- 鍾欣芳: field_worker → admin_staff, cross_group admin1
- Regenerate all 49 eval sheets with updated roles
- Add 兩人評分表.zip for download

https://claude.ai/code/session_01P9kqGzeEo3GNvL8KsQpiLU
</commit_message>
<xml_diff>
--- a/eval_output/品保課_周清家_評分表.xlsx
+++ b/eval_output/品保課_周清家_評分表.xlsx
@@ -1335,6 +1335,11 @@
           <t>劉祐誠</t>
         </is>
       </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>鍾欣芳</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="36" t="inlineStr">

</xml_diff>

<commit_message>
Fix 跨部門共評 to exclude non-admin roles
- 跨部門共評 evaluatees now limited to admin_staff and admin_group_leader
- Excludes: 班長, 組長, 副課長, 課長, 副理, 經理, 工程師
- 廠務部工程師 (曾夷璋, 陳家祥): new 'engineer' role, 部內共評 only
- Add engineer role handler in compute_evaluation_tasks

https://claude.ai/code/session_01P9kqGzeEo3GNvL8KsQpiLU
</commit_message>
<xml_diff>
--- a/eval_output/品保課_周清家_評分表.xlsx
+++ b/eval_output/品保課_周清家_評分表.xlsx
@@ -1247,95 +1247,70 @@
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>白惇維</t>
+          <t>王柳琦</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>王柳琦</t>
+          <t>徐惠蘭</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>徐惠蘭</t>
+          <t>沙洋</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>沙洋</t>
+          <t>石容瑄</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>曾夷璋</t>
+          <t>陳惠萍</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>陳家祥</t>
+          <t>尤念萍</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>王秀雯</t>
+          <t>林德和</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>石容瑄</t>
+          <t>羅文彥</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>陳惠萍</t>
+          <t>楊心恬</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>尤念萍</t>
+          <t>陳巧倫</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>林德和</t>
+          <t>郭惠婷</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>羅文彥</t>
+          <t>尤秐棠</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>楊心恬</t>
+          <t>陳孟怡</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
-        <is>
-          <t>陳巧倫</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>郭惠婷</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>尤秐棠</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>陳孟怡</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>劉祐誠</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
         <is>
           <t>鍾欣芳</t>
         </is>

</xml_diff>